<commit_message>
several changes upto saving project details
</commit_message>
<xml_diff>
--- a/api/templates/projects_import_template.xlsx
+++ b/api/templates/projects_import_template.xlsx
@@ -20,7 +20,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+  <si>
+    <t xml:space="preserve">ProjectRefNum</t>
+  </si>
   <si>
     <t xml:space="preserve">ProjectName</t>
   </si>
@@ -49,6 +52,18 @@
     <t xml:space="preserve"> implementing Agency</t>
   </si>
   <si>
+    <t xml:space="preserve">County</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constituency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ward</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MGD/01/2024</t>
+  </si>
+  <si>
     <t xml:space="preserve">Construction of ward North Seme office</t>
   </si>
   <si>
@@ -59,6 +74,15 @@
   </si>
   <si>
     <t xml:space="preserve">MOE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kesses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MailNe</t>
   </si>
 </sst>
 </file>
@@ -70,7 +94,7 @@
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="166" formatCode="mm/dd/yy"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -92,12 +116,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -142,16 +160,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -180,17 +194,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultColWidth="8.51953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr defaultColWidth="8.53125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="25.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="27.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1017" style="0" width="8.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="48.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="0" width="25.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="27.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1018" style="0" width="8.36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -211,40 +226,64 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="0" t="s">
         <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>9</v>
+      <c r="A2" s="0" t="s">
+        <v>13</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="E2" s="3" t="n">
         <v>45838</v>
-      </c>
-      <c r="E2" s="1" t="n">
-        <v>5000000</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>5000000</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" s="0" t="s">
-        <v>11</v>
+      <c r="G2" s="1" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>15</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>12</v>
+        <v>16</v>
+      </c>
+      <c r="J2" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="L2" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="M2" s="0" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Setting top menu defaults
</commit_message>
<xml_diff>
--- a/api/templates/projects_import_template.xlsx
+++ b/api/templates/projects_import_template.xlsx
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
-  <si>
-    <t xml:space="preserve">ProjectRefNum</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
   <si>
     <t xml:space="preserve">ProjectName</t>
   </si>
@@ -59,9 +56,6 @@
   </si>
   <si>
     <t xml:space="preserve">Ward</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MGD/01/2024</t>
   </si>
   <si>
     <t xml:space="preserve">Construction of ward North Seme office</t>
@@ -194,18 +188,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultColWidth="8.53125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="48.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="0" width="25.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="27.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1018" style="0" width="8.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="25.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="27.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1017" style="0" width="8.36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -226,13 +220,13 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="0" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="0" t="s">
@@ -241,49 +235,43 @@
       <c r="L1" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="0" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>13</v>
+      <c r="A2" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C2" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="D2" s="3" t="n">
         <v>45838</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>5000000</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>5000000</v>
       </c>
-      <c r="G2" s="1" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="H2" s="1" t="s">
+      <c r="G2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="J2" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="K2" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="L2" s="0" t="s">
         <v>18</v>
-      </c>
-      <c r="L2" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="M2" s="0" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>